<commit_message>
chore: sync Nova upm-release-2026.09.02-01
</commit_message>
<xml_diff>
--- a/Assets/Framework/Tracks/Tracks.xlsx
+++ b/Assets/Framework/Tracks/Tracks.xlsx
@@ -1,17 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowHeight="16660"/>
+    <workbookView windowWidth="29120" windowHeight="13200" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="$默认用户属性说明" sheetId="1" r:id="rId1"/>
     <sheet name="$公共事件属性说明" sheetId="2" r:id="rId2"/>
     <sheet name="$预置属性说明" sheetId="3" r:id="rId3"/>
     <sheet name="$注意事项" sheetId="4" r:id="rId4"/>
+    <sheet name="打点表-Network" sheetId="5" r:id="rId5"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'打点表-Network'!$A$1:$I$74</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -30,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="382" uniqueCount="235">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1048" uniqueCount="325">
   <si>
     <t>用户属性（TGA）</t>
   </si>
@@ -74,24 +78,7 @@
     <t>nova_openid</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="微软雅黑"/>
-        <charset val="134"/>
-      </rPr>
-      <t>第三方渠道登录后返回的</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <charset val="134"/>
-      </rPr>
-      <t>ID</t>
-    </r>
+    <t>第三方渠道登录后返回的ID</t>
   </si>
   <si>
     <t>set</t>
@@ -100,24 +87,7 @@
     <t>第三方渠道登录时上报</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="微软雅黑"/>
-        <charset val="134"/>
-      </rPr>
-      <t>第三方渠道登录后的</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <charset val="134"/>
-      </rPr>
-      <t>ID</t>
-    </r>
+    <t>第三方渠道登录后的ID</t>
   </si>
   <si>
     <t>nova_third_login_provider</t>
@@ -775,6 +745,276 @@
   </si>
   <si>
     <t>客户端SDK和TA系统会自动采集或生成一些属性，内容参考【预支属性说明】标签页</t>
+  </si>
+  <si>
+    <t>事件名</t>
+  </si>
+  <si>
+    <t>事件中文名</t>
+  </si>
+  <si>
+    <t>事件说明</t>
+  </si>
+  <si>
+    <t>属性名</t>
+  </si>
+  <si>
+    <t>属性说明</t>
+  </si>
+  <si>
+    <t>目标</t>
+  </si>
+  <si>
+    <t>uwr_request_start</t>
+  </si>
+  <si>
+    <t>UWR 请求链开始</t>
+  </si>
+  <si>
+    <t>一条逻辑请求链开始；单 URL 与主备/多轮/重试链均只上报一次。</t>
+  </si>
+  <si>
+    <t>uwr_schema_version</t>
+  </si>
+  <si>
+    <t>UWR 埋点 schema 版本，固定为 1。</t>
+  </si>
+  <si>
+    <t>首个候选发送前上报。</t>
+  </si>
+  <si>
+    <t>ITrackPlugin</t>
+  </si>
+  <si>
+    <t>固定 1 start → 0～N error → 1 end。</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>uwr_chain_id</t>
+  </si>
+  <si>
+    <t>一次逻辑请求链的关联 ID；同一条 start、零到多条 error、end 共用。</t>
+  </si>
+  <si>
+    <t>uwr_module</t>
+  </si>
+  <si>
+    <t>enum-string</t>
+  </si>
+  <si>
+    <t>产生请求的模块：app、asset 或 network。</t>
+  </si>
+  <si>
+    <t>uwr_operation_name</t>
+  </si>
+  <si>
+    <t>稳定操作名；不包含 query、请求体、请求头或其他敏感参数。</t>
+  </si>
+  <si>
+    <t>uwr_method</t>
+  </si>
+  <si>
+    <t>HTTP 方法的大写形式，例如 GET、POST。</t>
+  </si>
+  <si>
+    <t>uwr_scheme</t>
+  </si>
+  <si>
+    <t>当前物理发送 URL 的协议，例如 http 或 https。</t>
+  </si>
+  <si>
+    <t>uwr_host</t>
+  </si>
+  <si>
+    <t>当前事件对应物理发送使用的域名，可直接判断主备域名；不记录解析 IP。</t>
+  </si>
+  <si>
+    <t>uwr_port</t>
+  </si>
+  <si>
+    <t>当前 URL 的有效端口，含协议默认端口。</t>
+  </si>
+  <si>
+    <t>uwr_path</t>
+  </si>
+  <si>
+    <t>当前 URL 的 AbsolutePath，不包含 query 和 fragment。</t>
+  </si>
+  <si>
+    <t>uwr_request_timeout_sec</t>
+  </si>
+  <si>
+    <t>当前物理请求的超时秒数；App/Network 为请求超时，Asset Bundle 为 idle timeout，Asset .version 为 CheckTimeout，.hash/.bytes 为固定 60 秒。</t>
+  </si>
+  <si>
+    <t>uwr_retry_index</t>
+  </si>
+  <si>
+    <t>完整轮次组合的重试序号，从 0 开始；0 是首次执行，1 表示消耗第 1 次 RetryRequestCount/RetryDownloadCount。</t>
+  </si>
+  <si>
+    <t>uwr_round_index</t>
+  </si>
+  <si>
+    <t>当前重试周期内的完整候选轮次序号，从 0 开始。</t>
+  </si>
+  <si>
+    <t>uwr_candidate_index</t>
+  </si>
+  <si>
+    <t>当前轮内按实际执行顺序排列的候选序号，从 0 开始。</t>
+  </si>
+  <si>
+    <t>uwr_candidate_count</t>
+  </si>
+  <si>
+    <t>一轮内去重后的候选数量；通常主备齐全为 2，单 URL 为 1。</t>
+  </si>
+  <si>
+    <t>uwr_send_index</t>
+  </si>
+  <si>
+    <t>long</t>
+  </si>
+  <si>
+    <t>整条逻辑链内的物理发送序号，从 0 开始，跨轮次和重试周期递增。</t>
+  </si>
+  <si>
+    <t>uwr_network_reachability</t>
+  </si>
+  <si>
+    <t>Unity Application.internetReachability 的粗粒度状态；不证明目标域名实际可访问。</t>
+  </si>
+  <si>
+    <t>uwr_download_operation_id</t>
+  </si>
+  <si>
+    <t>仅 Asset：一次显式 Downloader 或元数据下载操作的关联 ID，可聚合同一操作下多个文件请求。</t>
+  </si>
+  <si>
+    <t>uwr_package</t>
+  </si>
+  <si>
+    <t>仅 Asset：YooAsset Package 名称。</t>
+  </si>
+  <si>
+    <t>uwr_file_type</t>
+  </si>
+  <si>
+    <t>仅 Asset：version、manifest_hash、manifest_bytes 或 bundle。</t>
+  </si>
+  <si>
+    <t>uwr_request_error</t>
+  </si>
+  <si>
+    <t>UWR 物理发送失败</t>
+  </si>
+  <si>
+    <t>当前物理发送失败且逻辑链需要记录异常；同一逻辑链可上报零到多条。</t>
+  </si>
+  <si>
+    <t>每个失败物理发送结束时最多上报一次。</t>
+  </si>
+  <si>
+    <t>主备切换、多轮和完整组合重试都保持同一 uwr_chain_id。</t>
+  </si>
+  <si>
+    <t>uwr_error_type</t>
+  </si>
+  <si>
+    <t>低基数错误大类：transport、timeout、http、data_processing、cancelled 或 exception。</t>
+  </si>
+  <si>
+    <t>uwr_leaf_error_code</t>
+  </si>
+  <si>
+    <t>最具体的稳定错误码；由 UWR 明确状态优先，错误文本仅作末级最佳努力分类。</t>
+  </si>
+  <si>
+    <t>uwr_status_code</t>
+  </si>
+  <si>
+    <t>收到正式 HTTP 响应时的状态码；未收到响应时不写。</t>
+  </si>
+  <si>
+    <t>uwr_send_elapsed_ms</t>
+  </si>
+  <si>
+    <t>当前物理发送耗时，单位毫秒。</t>
+  </si>
+  <si>
+    <t>uwr_downloaded_bytes</t>
+  </si>
+  <si>
+    <t>UWR 可可靠取得时记录当前物理发送已下载字节数；YooAsset 未暴露时不写。</t>
+  </si>
+  <si>
+    <t>uwr_total_bytes</t>
+  </si>
+  <si>
+    <t>Content-Length 等可靠来源可得时记录总字节数；未知时不写。</t>
+  </si>
+  <si>
+    <t>uwr_request_end</t>
+  </si>
+  <si>
+    <t>UWR 请求链结束</t>
+  </si>
+  <si>
+    <t>逻辑请求链最终结束，每条链只上报一次。</t>
+  </si>
+  <si>
+    <t>成功、不可继续的 HTTP 响应、取消或候选耗尽时上报。</t>
+  </si>
+  <si>
+    <t>通过坐标字段还原实际发送顺序；不存在整条链路总超时。</t>
+  </si>
+  <si>
+    <t>uwr_result</t>
+  </si>
+  <si>
+    <t>整条链最终结果：success、http_error、network_error、timeout、aborted、data_processing_error 或模块定义的稳定结果。</t>
+  </si>
+  <si>
+    <t>uwr_started_send_count</t>
+  </si>
+  <si>
+    <t>本逻辑链实际开始的物理发送总数。</t>
+  </si>
+  <si>
+    <t>uwr_recovered_by_retry</t>
+  </si>
+  <si>
+    <t>bool</t>
+  </si>
+  <si>
+    <t>最终成功且此前至少已有一次物理发送失败时为 true。</t>
+  </si>
+  <si>
+    <t>uwr_total_elapsed_ms</t>
+  </si>
+  <si>
+    <t>从 start 到 end 的整条逻辑链耗时，单位毫秒；不表示存在总超时限制。</t>
+  </si>
+  <si>
+    <t>失败终态的低基数错误大类；成功时不写。</t>
+  </si>
+  <si>
+    <t>失败终态最具体的稳定错误码；成功或无可用细分时不写。</t>
+  </si>
+  <si>
+    <t>最终候选收到正式 HTTP 响应时的状态码；未收到响应时不写。</t>
+  </si>
+  <si>
+    <t>最终一次物理发送耗时，单位毫秒。</t>
+  </si>
+  <si>
+    <t>UWR 可可靠取得时记录最终物理发送已下载字节数；YooAsset 未暴露时不写。</t>
+  </si>
+  <si>
+    <t>可靠来源可得时记录最终响应总字节数；未知时不写。</t>
   </si>
 </sst>
 </file>
@@ -787,10 +1027,17 @@
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="24">
+  <fonts count="25">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
       <charset val="134"/>
     </font>
@@ -966,12 +1213,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="36">
+  <fills count="37">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1F4E78"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -1178,7 +1431,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -1198,6 +1451,15 @@
       </top>
       <bottom style="thin">
         <color rgb="FFB7C7D6"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFD9E2F3"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1302,160 +1564,166 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="43" fontId="5" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="44" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="44" fontId="5" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="9" fontId="5" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="41" fontId="5" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="42" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="42" fontId="5" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="3">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="4">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="5">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="6">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="8" borderId="7">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="8" borderId="6">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="8" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="9" borderId="8">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="9">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="10">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="10" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="11" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="12" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="13" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="14" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="15" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="16" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="17" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="18" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="19" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="20" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="21" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="22" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="23" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="24" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="25" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="26" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="27" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="28" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="29" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="30" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="31" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="32" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="33" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="34" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="35" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="36" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -1778,275 +2046,275 @@
   <dimension ref="A1:F14"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8" outlineLevelCol="5"/>
   <cols>
-    <col min="1" max="1" width="28.2734375" customWidth="1"/>
-    <col min="2" max="2" width="26.7265625" customWidth="1"/>
-    <col min="3" max="4" width="10" customWidth="1"/>
-    <col min="5" max="5" width="24.546875" customWidth="1"/>
-    <col min="6" max="6" width="70.09375" customWidth="1"/>
+    <col min="1" max="1" width="28.2734375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="26.7265625" style="1" customWidth="1"/>
+    <col min="3" max="4" width="10" style="1" customWidth="1"/>
+    <col min="5" max="5" width="24.546875" style="1" customWidth="1"/>
+    <col min="6" max="6" width="70.09375" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="19.2" spans="1:6">
-      <c r="A1" s="1" t="s">
+    <row r="1" ht="19.2" customHeight="1" spans="1:6">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="2" spans="1:6">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="F2" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:6">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D3" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="E3" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="F3" s="6" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="4" ht="17" spans="1:6">
-      <c r="A4" s="3" t="s">
+    <row r="4" ht="17" customHeight="1" spans="1:6">
+      <c r="A4" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="E4" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="F4" s="4" t="s">
+      <c r="F4" s="6" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="5" spans="1:6">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D5" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="E5" s="5" t="s">
+      <c r="E5" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="F5" s="5" t="s">
+      <c r="F5" s="7" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="6" spans="1:6">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="D6" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="E6" s="3" t="s">
+      <c r="E6" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="F6" s="3" t="s">
+      <c r="F6" s="6" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="7" spans="1:6">
-      <c r="A7" s="3" t="s">
+      <c r="A7" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="C7" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="D7" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="E7" s="5" t="s">
+      <c r="E7" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="F7" s="5" t="s">
+      <c r="F7" s="7" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="8" spans="1:6">
-      <c r="A8" s="3" t="s">
+      <c r="A8" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="C8" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="D8" s="3" t="s">
+      <c r="D8" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="E8" s="5" t="s">
+      <c r="E8" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="F8" s="5" t="s">
+      <c r="F8" s="7" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="9" spans="1:6">
-      <c r="A9" s="3" t="s">
+      <c r="A9" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="B9" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="C9" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="D9" s="3" t="s">
+      <c r="D9" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="E9" s="5" t="s">
+      <c r="E9" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="F9" s="5" t="s">
+      <c r="F9" s="7" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="10" spans="1:6">
-      <c r="A10" s="3" t="s">
+      <c r="A10" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="B10" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="C10" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="D10" s="3" t="s">
+      <c r="D10" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="E10" s="5" t="s">
+      <c r="E10" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="F10" s="5" t="s">
+      <c r="F10" s="7" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="11" spans="1:6">
-      <c r="A11" s="3" t="s">
+      <c r="A11" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="B11" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="C11" s="3" t="s">
+      <c r="C11" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="D11" s="3" t="s">
+      <c r="D11" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="E11" s="5" t="s">
+      <c r="E11" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="F11" s="5" t="s">
+      <c r="F11" s="7" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="12" spans="1:6">
-      <c r="A12" s="3" t="s">
+      <c r="A12" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="B12" s="5" t="s">
+      <c r="B12" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="C12" s="3" t="s">
+      <c r="C12" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="D12" s="3" t="s">
+      <c r="D12" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="E12" s="5" t="s">
+      <c r="E12" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="F12" s="5" t="s">
+      <c r="F12" s="7" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="13" spans="1:6">
-      <c r="A13" s="3" t="s">
+      <c r="A13" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="B13" s="5" t="s">
+      <c r="B13" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="C13" s="3" t="s">
+      <c r="C13" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="D13" s="3" t="s">
+      <c r="D13" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="E13" s="5" t="s">
+      <c r="E13" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="F13" s="5" t="s">
+      <c r="F13" s="7" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="14" spans="1:6">
-      <c r="A14" s="3" t="s">
+      <c r="A14" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="B14" s="5" t="s">
+      <c r="B14" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="C14" s="3" t="s">
+      <c r="C14" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="D14" s="3" t="s">
+      <c r="D14" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="E14" s="5" t="s">
+      <c r="E14" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="F14" s="5" t="s">
+      <c r="F14" s="7" t="s">
         <v>52</v>
       </c>
     </row>
@@ -2063,56 +2331,56 @@
   <dimension ref="A1:F3"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8" outlineLevelRow="2" outlineLevelCol="5"/>
   <cols>
-    <col min="1" max="1" width="20" customWidth="1"/>
-    <col min="2" max="2" width="13" customWidth="1"/>
-    <col min="3" max="3" width="10" customWidth="1"/>
-    <col min="4" max="4" width="18" customWidth="1"/>
-    <col min="5" max="5" width="24" customWidth="1"/>
-    <col min="6" max="6" width="16" customWidth="1"/>
+    <col min="1" max="1" width="20" style="1" customWidth="1"/>
+    <col min="2" max="2" width="13" style="1" customWidth="1"/>
+    <col min="3" max="3" width="10" style="1" customWidth="1"/>
+    <col min="4" max="4" width="18" style="1" customWidth="1"/>
+    <col min="5" max="5" width="24" style="1" customWidth="1"/>
+    <col min="6" max="6" width="16" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="19.2" spans="1:6">
-      <c r="A1" s="1" t="s">
+    <row r="1" ht="19.2" customHeight="1" spans="1:6">
+      <c r="A1" s="4" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="2" spans="1:6">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="F2" s="5" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="3" spans="1:6">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D3" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="E3" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="F3" s="6" t="s">
         <v>62</v>
       </c>
     </row>
@@ -2129,933 +2397,933 @@
   <dimension ref="A1:E55"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8" outlineLevelCol="4"/>
   <cols>
-    <col min="1" max="1" width="15" customWidth="1"/>
-    <col min="2" max="2" width="25" customWidth="1"/>
-    <col min="3" max="3" width="16" customWidth="1"/>
-    <col min="4" max="4" width="55" customWidth="1"/>
-    <col min="5" max="5" width="19" customWidth="1"/>
+    <col min="1" max="1" width="15" style="1" customWidth="1"/>
+    <col min="2" max="2" width="25" style="1" customWidth="1"/>
+    <col min="3" max="3" width="16" style="1" customWidth="1"/>
+    <col min="4" max="4" width="55" style="1" customWidth="1"/>
+    <col min="5" max="5" width="19" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="19.2" spans="1:5">
-      <c r="A1" s="1" t="s">
+    <row r="1" ht="19.2" customHeight="1" spans="1:5">
+      <c r="A1" s="4" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="5" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="3" spans="1:5">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D3" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="E3" s="6" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="6" t="s">
         <v>69</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E4" s="6" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="5" spans="1:5">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="6" t="s">
         <v>73</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D5" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="E5" s="6" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="6" spans="1:5">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="6" t="s">
         <v>75</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" s="6" t="s">
         <v>76</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="D6" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="E6" s="3" t="s">
+      <c r="E6" s="6" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="7" spans="1:5">
-      <c r="A7" s="3" t="s">
+      <c r="A7" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="C7" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="D7" s="6" t="s">
         <v>80</v>
       </c>
-      <c r="E7" s="3" t="s">
+      <c r="E7" s="6" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="8" spans="1:5">
-      <c r="A8" s="3" t="s">
+      <c r="A8" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="B8" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="C8" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="D8" s="3" t="s">
+      <c r="D8" s="6" t="s">
         <v>83</v>
       </c>
-      <c r="E8" s="3" t="s">
+      <c r="E8" s="6" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="9" spans="1:5">
-      <c r="A9" s="3" t="s">
+      <c r="A9" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="B9" s="6" t="s">
         <v>84</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="C9" s="6" t="s">
         <v>85</v>
       </c>
-      <c r="D9" s="3" t="s">
+      <c r="D9" s="6" t="s">
         <v>86</v>
       </c>
-      <c r="E9" s="3" t="s">
+      <c r="E9" s="6" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="10" spans="1:5">
-      <c r="A10" s="3" t="s">
+      <c r="A10" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="B10" s="6" t="s">
         <v>87</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="C10" s="6" t="s">
         <v>88</v>
       </c>
-      <c r="D10" s="3" t="s">
+      <c r="D10" s="6" t="s">
         <v>89</v>
       </c>
-      <c r="E10" s="3" t="s">
+      <c r="E10" s="6" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="11" spans="1:5">
-      <c r="A11" s="3" t="s">
+      <c r="A11" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="B11" s="3" t="s">
+      <c r="B11" s="6" t="s">
         <v>91</v>
       </c>
-      <c r="C11" s="3" t="s">
+      <c r="C11" s="6" t="s">
         <v>92</v>
       </c>
-      <c r="D11" s="3" t="s">
+      <c r="D11" s="6" t="s">
         <v>93</v>
       </c>
-      <c r="E11" s="3" t="s">
+      <c r="E11" s="6" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="12" spans="1:5">
-      <c r="A12" s="3" t="s">
+      <c r="A12" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="B12" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="C12" s="3" t="s">
+      <c r="C12" s="6" t="s">
         <v>96</v>
       </c>
-      <c r="D12" s="3" t="s">
+      <c r="D12" s="6" t="s">
         <v>97</v>
       </c>
-      <c r="E12" s="3" t="s">
+      <c r="E12" s="6" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="13" spans="1:5">
-      <c r="A13" s="3" t="s">
+      <c r="A13" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="B13" s="3" t="s">
+      <c r="B13" s="6" t="s">
         <v>98</v>
       </c>
-      <c r="C13" s="3" t="s">
+      <c r="C13" s="6" t="s">
         <v>99</v>
       </c>
-      <c r="D13" s="3" t="s">
+      <c r="D13" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="E13" s="3" t="s">
+      <c r="E13" s="6" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="14" spans="1:5">
-      <c r="A14" s="3" t="s">
+      <c r="A14" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="B14" s="3" t="s">
+      <c r="B14" s="6" t="s">
         <v>101</v>
       </c>
-      <c r="C14" s="3" t="s">
+      <c r="C14" s="6" t="s">
         <v>102</v>
       </c>
-      <c r="D14" s="3" t="s">
+      <c r="D14" s="6" t="s">
         <v>103</v>
       </c>
-      <c r="E14" s="3" t="s">
+      <c r="E14" s="6" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="15" spans="1:5">
-      <c r="A15" s="3" t="s">
+      <c r="A15" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="B15" s="3" t="s">
+      <c r="B15" s="6" t="s">
         <v>104</v>
       </c>
-      <c r="C15" s="3" t="s">
+      <c r="C15" s="6" t="s">
         <v>105</v>
       </c>
-      <c r="D15" s="3" t="s">
+      <c r="D15" s="6" t="s">
         <v>106</v>
       </c>
-      <c r="E15" s="3" t="s">
+      <c r="E15" s="6" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="16" spans="1:5">
-      <c r="A16" s="3" t="s">
+      <c r="A16" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="B16" s="3" t="s">
+      <c r="B16" s="6" t="s">
         <v>107</v>
       </c>
-      <c r="C16" s="3" t="s">
+      <c r="C16" s="6" t="s">
         <v>108</v>
       </c>
-      <c r="D16" s="3" t="s">
+      <c r="D16" s="6" t="s">
         <v>109</v>
       </c>
-      <c r="E16" s="3" t="s">
+      <c r="E16" s="6" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="17" spans="1:5">
-      <c r="A17" s="3" t="s">
+      <c r="A17" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="B17" s="3" t="s">
+      <c r="B17" s="6" t="s">
         <v>110</v>
       </c>
-      <c r="C17" s="3" t="s">
+      <c r="C17" s="6" t="s">
         <v>111</v>
       </c>
-      <c r="D17" s="3" t="s">
+      <c r="D17" s="6" t="s">
         <v>112</v>
       </c>
-      <c r="E17" s="3" t="s">
+      <c r="E17" s="6" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="18" spans="1:5">
-      <c r="A18" s="3" t="s">
+      <c r="A18" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="B18" s="3" t="s">
+      <c r="B18" s="6" t="s">
         <v>113</v>
       </c>
-      <c r="C18" s="3" t="s">
+      <c r="C18" s="6" t="s">
         <v>114</v>
       </c>
-      <c r="D18" s="3" t="s">
+      <c r="D18" s="6" t="s">
         <v>115</v>
       </c>
-      <c r="E18" s="3" t="s">
+      <c r="E18" s="6" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="19" spans="1:5">
-      <c r="A19" s="3" t="s">
+      <c r="A19" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="B19" s="3" t="s">
+      <c r="B19" s="6" t="s">
         <v>116</v>
       </c>
-      <c r="C19" s="3" t="s">
+      <c r="C19" s="6" t="s">
         <v>117</v>
       </c>
-      <c r="D19" s="3" t="s">
+      <c r="D19" s="6" t="s">
         <v>118</v>
       </c>
-      <c r="E19" s="3" t="s">
+      <c r="E19" s="6" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="20" spans="1:5">
-      <c r="A20" s="3" t="s">
+      <c r="A20" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="B20" s="3" t="s">
+      <c r="B20" s="6" t="s">
         <v>119</v>
       </c>
-      <c r="C20" s="3" t="s">
+      <c r="C20" s="6" t="s">
         <v>120</v>
       </c>
-      <c r="D20" s="3" t="s">
+      <c r="D20" s="6" t="s">
         <v>121</v>
       </c>
-      <c r="E20" s="3" t="s">
+      <c r="E20" s="6" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="21" spans="1:5">
-      <c r="A21" s="3" t="s">
+      <c r="A21" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="B21" s="3" t="s">
+      <c r="B21" s="6" t="s">
         <v>122</v>
       </c>
-      <c r="C21" s="3" t="s">
+      <c r="C21" s="6" t="s">
         <v>123</v>
       </c>
-      <c r="D21" s="3" t="s">
+      <c r="D21" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="E21" s="3" t="s">
+      <c r="E21" s="6" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="22" spans="1:5">
-      <c r="A22" s="3" t="s">
+      <c r="A22" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="B22" s="3" t="s">
+      <c r="B22" s="6" t="s">
         <v>125</v>
       </c>
-      <c r="C22" s="3" t="s">
+      <c r="C22" s="6" t="s">
         <v>126</v>
       </c>
-      <c r="D22" s="3" t="s">
+      <c r="D22" s="6" t="s">
         <v>127</v>
       </c>
-      <c r="E22" s="3" t="s">
+      <c r="E22" s="6" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="23" spans="1:5">
-      <c r="A23" s="3" t="s">
+      <c r="A23" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="B23" s="3" t="s">
+      <c r="B23" s="6" t="s">
         <v>128</v>
       </c>
-      <c r="C23" s="3" t="s">
+      <c r="C23" s="6" t="s">
         <v>129</v>
       </c>
-      <c r="D23" s="3" t="s">
+      <c r="D23" s="6" t="s">
         <v>130</v>
       </c>
-      <c r="E23" s="3" t="s">
+      <c r="E23" s="6" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="24" spans="1:5">
-      <c r="A24" s="3" t="s">
+      <c r="A24" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="B24" s="3" t="s">
+      <c r="B24" s="6" t="s">
         <v>131</v>
       </c>
-      <c r="C24" s="3" t="s">
+      <c r="C24" s="6" t="s">
         <v>132</v>
       </c>
-      <c r="D24" s="3" t="s">
+      <c r="D24" s="6" t="s">
         <v>133</v>
       </c>
-      <c r="E24" s="3" t="s">
+      <c r="E24" s="6" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="25" spans="1:5">
-      <c r="A25" s="3" t="s">
+      <c r="A25" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="B25" s="3" t="s">
+      <c r="B25" s="6" t="s">
         <v>134</v>
       </c>
-      <c r="C25" s="3" t="s">
+      <c r="C25" s="6" t="s">
         <v>135</v>
       </c>
-      <c r="D25" s="3" t="s">
+      <c r="D25" s="6" t="s">
         <v>136</v>
       </c>
-      <c r="E25" s="3" t="s">
+      <c r="E25" s="6" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="26" spans="1:5">
-      <c r="A26" s="3" t="s">
+      <c r="A26" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="B26" s="3" t="s">
+      <c r="B26" s="6" t="s">
         <v>137</v>
       </c>
-      <c r="C26" s="3" t="s">
+      <c r="C26" s="6" t="s">
         <v>138</v>
       </c>
-      <c r="D26" s="3" t="s">
+      <c r="D26" s="6" t="s">
         <v>139</v>
       </c>
-      <c r="E26" s="3" t="s">
+      <c r="E26" s="6" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="27" spans="1:5">
-      <c r="A27" s="3" t="s">
+      <c r="A27" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="B27" s="3" t="s">
+      <c r="B27" s="6" t="s">
         <v>140</v>
       </c>
-      <c r="C27" s="3" t="s">
+      <c r="C27" s="6" t="s">
         <v>141</v>
       </c>
-      <c r="D27" s="3" t="s">
+      <c r="D27" s="6" t="s">
         <v>142</v>
       </c>
-      <c r="E27" s="3" t="s">
+      <c r="E27" s="6" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="28" spans="1:5">
-      <c r="A28" s="3" t="s">
+      <c r="A28" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="B28" s="3" t="s">
+      <c r="B28" s="6" t="s">
         <v>143</v>
       </c>
-      <c r="C28" s="3" t="s">
+      <c r="C28" s="6" t="s">
         <v>144</v>
       </c>
-      <c r="D28" s="3" t="s">
+      <c r="D28" s="6" t="s">
         <v>145</v>
       </c>
-      <c r="E28" s="3" t="s">
+      <c r="E28" s="6" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="29" spans="1:5">
-      <c r="A29" s="3" t="s">
+      <c r="A29" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="B29" s="3" t="s">
+      <c r="B29" s="6" t="s">
         <v>146</v>
       </c>
-      <c r="C29" s="3" t="s">
+      <c r="C29" s="6" t="s">
         <v>147</v>
       </c>
-      <c r="D29" s="3" t="s">
+      <c r="D29" s="6" t="s">
         <v>148</v>
       </c>
-      <c r="E29" s="3" t="s">
+      <c r="E29" s="6" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="30" spans="1:5">
-      <c r="A30" s="3" t="s">
+      <c r="A30" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="B30" s="3" t="s">
+      <c r="B30" s="6" t="s">
         <v>149</v>
       </c>
-      <c r="C30" s="3" t="s">
+      <c r="C30" s="6" t="s">
         <v>150</v>
       </c>
-      <c r="D30" s="3" t="s">
+      <c r="D30" s="6" t="s">
         <v>151</v>
       </c>
-      <c r="E30" s="3" t="s">
+      <c r="E30" s="6" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="31" spans="1:5">
-      <c r="A31" s="3" t="s">
+      <c r="A31" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="B31" s="3" t="s">
+      <c r="B31" s="6" t="s">
         <v>152</v>
       </c>
-      <c r="C31" s="3" t="s">
+      <c r="C31" s="6" t="s">
         <v>153</v>
       </c>
-      <c r="D31" s="3" t="s">
+      <c r="D31" s="6" t="s">
         <v>154</v>
       </c>
-      <c r="E31" s="3" t="s">
+      <c r="E31" s="6" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="32" spans="1:5">
-      <c r="A32" s="3" t="s">
+      <c r="A32" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="B32" s="3" t="s">
+      <c r="B32" s="6" t="s">
         <v>155</v>
       </c>
-      <c r="C32" s="3" t="s">
+      <c r="C32" s="6" t="s">
         <v>156</v>
       </c>
-      <c r="D32" s="3" t="s">
+      <c r="D32" s="6" t="s">
         <v>157</v>
       </c>
-      <c r="E32" s="3" t="s">
+      <c r="E32" s="6" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="33" spans="1:5">
-      <c r="A33" s="3" t="s">
+      <c r="A33" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="B33" s="3" t="s">
+      <c r="B33" s="6" t="s">
         <v>158</v>
       </c>
-      <c r="C33" s="3" t="s">
+      <c r="C33" s="6" t="s">
         <v>159</v>
       </c>
-      <c r="D33" s="3" t="s">
+      <c r="D33" s="6" t="s">
         <v>160</v>
       </c>
-      <c r="E33" s="3" t="s">
+      <c r="E33" s="6" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="34" spans="1:5">
-      <c r="A34" s="3" t="s">
+      <c r="A34" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="B34" s="3" t="s">
+      <c r="B34" s="6" t="s">
         <v>161</v>
       </c>
-      <c r="C34" s="3" t="s">
+      <c r="C34" s="6" t="s">
         <v>162</v>
       </c>
-      <c r="D34" s="3" t="s">
+      <c r="D34" s="6" t="s">
         <v>163</v>
       </c>
-      <c r="E34" s="3" t="s">
+      <c r="E34" s="6" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="35" spans="1:5">
-      <c r="A35" s="3" t="s">
+      <c r="A35" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="B35" s="3" t="s">
+      <c r="B35" s="6" t="s">
         <v>164</v>
       </c>
-      <c r="C35" s="3" t="s">
+      <c r="C35" s="6" t="s">
         <v>165</v>
       </c>
-      <c r="D35" s="3" t="s">
+      <c r="D35" s="6" t="s">
         <v>166</v>
       </c>
-      <c r="E35" s="3" t="s">
+      <c r="E35" s="6" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="36" spans="1:5">
-      <c r="A36" s="3" t="s">
+      <c r="A36" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="B36" s="3" t="s">
+      <c r="B36" s="6" t="s">
         <v>167</v>
       </c>
-      <c r="C36" s="3" t="s">
+      <c r="C36" s="6" t="s">
         <v>168</v>
       </c>
-      <c r="D36" s="3" t="s">
+      <c r="D36" s="6" t="s">
         <v>169</v>
       </c>
-      <c r="E36" s="3" t="s">
+      <c r="E36" s="6" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="37" spans="1:5">
-      <c r="A37" s="3" t="s">
+      <c r="A37" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="B37" s="3" t="s">
+      <c r="B37" s="6" t="s">
         <v>170</v>
       </c>
-      <c r="C37" s="3" t="s">
+      <c r="C37" s="6" t="s">
         <v>171</v>
       </c>
-      <c r="D37" s="3" t="s">
+      <c r="D37" s="6" t="s">
         <v>172</v>
       </c>
-      <c r="E37" s="3" t="s">
+      <c r="E37" s="6" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="38" spans="1:5">
-      <c r="A38" s="3" t="s">
+      <c r="A38" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="B38" s="3" t="s">
+      <c r="B38" s="6" t="s">
         <v>173</v>
       </c>
-      <c r="C38" s="3" t="s">
+      <c r="C38" s="6" t="s">
         <v>174</v>
       </c>
-      <c r="D38" s="3" t="s">
+      <c r="D38" s="6" t="s">
         <v>175</v>
       </c>
-      <c r="E38" s="3" t="s">
+      <c r="E38" s="6" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="39" spans="1:5">
-      <c r="A39" s="3" t="s">
+      <c r="A39" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="B39" s="3" t="s">
+      <c r="B39" s="6" t="s">
         <v>176</v>
       </c>
-      <c r="C39" s="3" t="s">
+      <c r="C39" s="6" t="s">
         <v>177</v>
       </c>
-      <c r="D39" s="3" t="s">
+      <c r="D39" s="6" t="s">
         <v>178</v>
       </c>
-      <c r="E39" s="3" t="s">
+      <c r="E39" s="6" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="40" spans="1:5">
-      <c r="A40" s="3" t="s">
+      <c r="A40" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="B40" s="3" t="s">
+      <c r="B40" s="6" t="s">
         <v>179</v>
       </c>
-      <c r="C40" s="3" t="s">
+      <c r="C40" s="6" t="s">
         <v>180</v>
       </c>
-      <c r="D40" s="3" t="s">
+      <c r="D40" s="6" t="s">
         <v>181</v>
       </c>
-      <c r="E40" s="3" t="s">
+      <c r="E40" s="6" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="41" spans="1:5">
-      <c r="A41" s="3" t="s">
+      <c r="A41" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="B41" s="3" t="s">
+      <c r="B41" s="6" t="s">
         <v>182</v>
       </c>
-      <c r="C41" s="3" t="s">
+      <c r="C41" s="6" t="s">
         <v>183</v>
       </c>
-      <c r="D41" s="3" t="s">
+      <c r="D41" s="6" t="s">
         <v>184</v>
       </c>
-      <c r="E41" s="3" t="s">
+      <c r="E41" s="6" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="42" spans="1:5">
-      <c r="A42" s="3" t="s">
+      <c r="A42" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="B42" s="3" t="s">
+      <c r="B42" s="6" t="s">
         <v>185</v>
       </c>
-      <c r="C42" s="3" t="s">
+      <c r="C42" s="6" t="s">
         <v>186</v>
       </c>
-      <c r="D42" s="3" t="s">
+      <c r="D42" s="6" t="s">
         <v>187</v>
       </c>
-      <c r="E42" s="3" t="s">
+      <c r="E42" s="6" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="43" spans="1:5">
-      <c r="A43" s="3" t="s">
+      <c r="A43" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="B43" s="3" t="s">
+      <c r="B43" s="6" t="s">
         <v>188</v>
       </c>
-      <c r="C43" s="3" t="s">
+      <c r="C43" s="6" t="s">
         <v>189</v>
       </c>
-      <c r="D43" s="3" t="s">
+      <c r="D43" s="6" t="s">
         <v>190</v>
       </c>
-      <c r="E43" s="3" t="s">
+      <c r="E43" s="6" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="44" spans="1:5">
-      <c r="A44" s="3" t="s">
+      <c r="A44" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="B44" s="3" t="s">
+      <c r="B44" s="6" t="s">
         <v>191</v>
       </c>
-      <c r="C44" s="3" t="s">
+      <c r="C44" s="6" t="s">
         <v>192</v>
       </c>
-      <c r="D44" s="3" t="s">
+      <c r="D44" s="6" t="s">
         <v>193</v>
       </c>
-      <c r="E44" s="3" t="s">
+      <c r="E44" s="6" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="45" spans="1:5">
-      <c r="A45" s="3" t="s">
+      <c r="A45" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="B45" s="3" t="s">
+      <c r="B45" s="6" t="s">
         <v>194</v>
       </c>
-      <c r="C45" s="3" t="s">
+      <c r="C45" s="6" t="s">
         <v>195</v>
       </c>
-      <c r="D45" s="3" t="s">
+      <c r="D45" s="6" t="s">
         <v>196</v>
       </c>
-      <c r="E45" s="3" t="s">
+      <c r="E45" s="6" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="46" spans="1:5">
-      <c r="A46" s="3" t="s">
+      <c r="A46" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="B46" s="3" t="s">
+      <c r="B46" s="6" t="s">
         <v>197</v>
       </c>
-      <c r="C46" s="3" t="s">
+      <c r="C46" s="6" t="s">
         <v>198</v>
       </c>
-      <c r="D46" s="3" t="s">
+      <c r="D46" s="6" t="s">
         <v>199</v>
       </c>
-      <c r="E46" s="3" t="s">
+      <c r="E46" s="6" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="47" spans="1:5">
-      <c r="A47" s="3" t="s">
+      <c r="A47" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="B47" s="3" t="s">
+      <c r="B47" s="6" t="s">
         <v>200</v>
       </c>
-      <c r="C47" s="3" t="s">
+      <c r="C47" s="6" t="s">
         <v>201</v>
       </c>
-      <c r="D47" s="3" t="s">
+      <c r="D47" s="6" t="s">
         <v>202</v>
       </c>
-      <c r="E47" s="3" t="s">
+      <c r="E47" s="6" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="48" spans="1:5">
-      <c r="A48" s="3" t="s">
+      <c r="A48" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="B48" s="3" t="s">
+      <c r="B48" s="6" t="s">
         <v>203</v>
       </c>
-      <c r="C48" s="3" t="s">
+      <c r="C48" s="6" t="s">
         <v>204</v>
       </c>
-      <c r="D48" s="3" t="s">
+      <c r="D48" s="6" t="s">
         <v>205</v>
       </c>
-      <c r="E48" s="3" t="s">
+      <c r="E48" s="6" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="49" spans="1:5">
-      <c r="A49" s="3" t="s">
+      <c r="A49" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="B49" s="3" t="s">
+      <c r="B49" s="6" t="s">
         <v>206</v>
       </c>
-      <c r="C49" s="3" t="s">
+      <c r="C49" s="6" t="s">
         <v>207</v>
       </c>
-      <c r="D49" s="3" t="s">
+      <c r="D49" s="6" t="s">
         <v>208</v>
       </c>
-      <c r="E49" s="3" t="s">
+      <c r="E49" s="6" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="50" spans="1:5">
-      <c r="A50" s="3" t="s">
+      <c r="A50" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="B50" s="3" t="s">
+      <c r="B50" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="C50" s="3" t="s">
+      <c r="C50" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="D50" s="3" t="s">
+      <c r="D50" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="E50" s="3" t="s">
+      <c r="E50" s="6" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="51" spans="1:5">
-      <c r="A51" s="3" t="s">
+      <c r="A51" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="B51" s="3" t="s">
+      <c r="B51" s="6" t="s">
         <v>69</v>
       </c>
-      <c r="C51" s="3" t="s">
+      <c r="C51" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="D51" s="3" t="s">
+      <c r="D51" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="E51" s="3" t="s">
+      <c r="E51" s="6" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="52" spans="1:5">
-      <c r="A52" s="3" t="s">
+      <c r="A52" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="B52" s="3" t="s">
+      <c r="B52" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="C52" s="3" t="s">
+      <c r="C52" s="6" t="s">
         <v>73</v>
       </c>
-      <c r="D52" s="3" t="s">
+      <c r="D52" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="E52" s="3" t="s">
+      <c r="E52" s="6" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="53" spans="1:5">
-      <c r="A53" s="3" t="s">
+      <c r="A53" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="B53" s="3" t="s">
+      <c r="B53" s="6" t="s">
         <v>209</v>
       </c>
-      <c r="C53" s="3" t="s">
+      <c r="C53" s="6" t="s">
         <v>210</v>
       </c>
-      <c r="D53" s="3" t="s">
+      <c r="D53" s="6" t="s">
         <v>211</v>
       </c>
-      <c r="E53" s="3" t="s">
+      <c r="E53" s="6" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="54" spans="1:5">
-      <c r="A54" s="3" t="s">
+      <c r="A54" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="B54" s="3" t="s">
+      <c r="B54" s="6" t="s">
         <v>212</v>
       </c>
-      <c r="C54" s="3" t="s">
+      <c r="C54" s="6" t="s">
         <v>213</v>
       </c>
-      <c r="D54" s="3" t="s">
+      <c r="D54" s="6" t="s">
         <v>214</v>
       </c>
-      <c r="E54" s="3" t="s">
+      <c r="E54" s="6" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="55" spans="1:5">
-      <c r="A55" s="3" t="s">
+      <c r="A55" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="B55" s="3" t="s">
+      <c r="B55" s="6" t="s">
         <v>87</v>
       </c>
-      <c r="C55" s="3" t="s">
+      <c r="C55" s="6" t="s">
         <v>88</v>
       </c>
-      <c r="D55" s="3" t="s">
+      <c r="D55" s="6" t="s">
         <v>215</v>
       </c>
-      <c r="E55" s="3" t="s">
+      <c r="E55" s="6" t="s">
         <v>68</v>
       </c>
     </row>
@@ -3071,84 +3339,84 @@
   <dimension ref="A1:B10"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8" outlineLevelCol="1"/>
   <cols>
-    <col min="1" max="1" width="15" customWidth="1"/>
-    <col min="2" max="2" width="55" customWidth="1"/>
+    <col min="1" max="1" width="15" style="1" customWidth="1"/>
+    <col min="2" max="2" width="55" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="19.2" spans="1:2">
-      <c r="A1" s="1" t="s">
+    <row r="1" ht="19.2" customHeight="1" spans="1:2">
+      <c r="A1" s="4" t="s">
         <v>216</v>
       </c>
     </row>
     <row r="2" spans="1:2">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="5" t="s">
         <v>217</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="5" t="s">
         <v>218</v>
       </c>
     </row>
     <row r="3" spans="1:2">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="6" t="s">
         <v>219</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="6" t="s">
         <v>220</v>
       </c>
     </row>
     <row r="4" spans="1:2">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="6" t="s">
         <v>221</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="6" t="s">
         <v>222</v>
       </c>
     </row>
     <row r="5" spans="1:2">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="6" t="s">
         <v>223</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="6" t="s">
         <v>224</v>
       </c>
     </row>
     <row r="6" spans="1:2">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="6" t="s">
         <v>225</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="6" t="s">
         <v>226</v>
       </c>
     </row>
     <row r="7" spans="1:2">
-      <c r="A7" s="3" t="s">
+      <c r="A7" s="6" t="s">
         <v>227</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="6" t="s">
         <v>228</v>
       </c>
     </row>
     <row r="8" spans="1:2">
-      <c r="A8" s="3" t="s">
+      <c r="A8" s="6" t="s">
         <v>229</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="B8" s="6" t="s">
         <v>230</v>
       </c>
     </row>
     <row r="9" spans="1:2">
-      <c r="A9" s="3" t="s">
+      <c r="A9" s="6" t="s">
         <v>231</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="B9" s="6" t="s">
         <v>232</v>
       </c>
     </row>
     <row r="10" spans="1:2">
-      <c r="A10" s="3" t="s">
+      <c r="A10" s="6" t="s">
         <v>233</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="B10" s="6" t="s">
         <v>234</v>
       </c>
     </row>
@@ -3156,4 +3424,2176 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:I74"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8"/>
+  <cols>
+    <col min="1" max="1" width="28" style="1" customWidth="1"/>
+    <col min="2" max="2" width="18" style="1" customWidth="1"/>
+    <col min="3" max="3" width="36" style="1" customWidth="1"/>
+    <col min="4" max="4" width="40" style="1" customWidth="1"/>
+    <col min="5" max="5" width="14" style="1" customWidth="1"/>
+    <col min="6" max="6" width="58" style="1" customWidth="1"/>
+    <col min="7" max="7" width="32" style="1" customWidth="1"/>
+    <col min="8" max="8" width="16" style="1" customWidth="1"/>
+    <col min="9" max="9" width="48" style="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="17" spans="1:9">
+      <c r="A1" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>236</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>238</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" ht="34" spans="1:9">
+      <c r="A2" s="3" t="s">
+        <v>241</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>242</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>243</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>244</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>245</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>246</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="3" ht="30" customHeight="1" spans="1:9">
+      <c r="A3" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>250</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>251</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="I3" s="3" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1" spans="1:9">
+      <c r="A4" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>252</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>253</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>254</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="I4" s="3" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1" spans="1:9">
+      <c r="A5" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>255</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>256</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="H5" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="I5" s="3" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1" spans="1:9">
+      <c r="A6" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>257</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>258</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="H6" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="I6" s="3" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1" spans="1:9">
+      <c r="A7" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>259</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>260</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="H7" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="I7" s="3" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1" spans="1:9">
+      <c r="A8" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>261</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>262</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="H8" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="I8" s="3" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1" spans="1:9">
+      <c r="A9" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>263</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>264</v>
+      </c>
+      <c r="G9" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="H9" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="I9" s="3" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1" spans="1:9">
+      <c r="A10" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>265</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>266</v>
+      </c>
+      <c r="G10" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="H10" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="I10" s="3" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1" spans="1:9">
+      <c r="A11" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>267</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>268</v>
+      </c>
+      <c r="G11" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="H11" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="I11" s="3" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="12" ht="30" customHeight="1" spans="1:9">
+      <c r="A12" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>269</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>270</v>
+      </c>
+      <c r="G12" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="H12" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="I12" s="3" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="13" ht="30" customHeight="1" spans="1:9">
+      <c r="A13" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>271</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="F13" s="3" t="s">
+        <v>272</v>
+      </c>
+      <c r="G13" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="H13" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="I13" s="3" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="14" ht="30" customHeight="1" spans="1:9">
+      <c r="A14" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>273</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>274</v>
+      </c>
+      <c r="G14" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="H14" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="I14" s="3" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="15" ht="30" customHeight="1" spans="1:9">
+      <c r="A15" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>275</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="F15" s="3" t="s">
+        <v>276</v>
+      </c>
+      <c r="G15" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="H15" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="I15" s="3" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="16" ht="30" customHeight="1" spans="1:9">
+      <c r="A16" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>277</v>
+      </c>
+      <c r="E16" s="3" t="s">
+        <v>278</v>
+      </c>
+      <c r="F16" s="3" t="s">
+        <v>279</v>
+      </c>
+      <c r="G16" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="H16" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="I16" s="3" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="17" ht="30" customHeight="1" spans="1:9">
+      <c r="A17" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>280</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>253</v>
+      </c>
+      <c r="F17" s="3" t="s">
+        <v>281</v>
+      </c>
+      <c r="G17" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="H17" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="I17" s="3" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="18" ht="30" customHeight="1" spans="1:9">
+      <c r="A18" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>282</v>
+      </c>
+      <c r="E18" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F18" s="3" t="s">
+        <v>283</v>
+      </c>
+      <c r="G18" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="H18" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="I18" s="3" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="19" ht="30" customHeight="1" spans="1:9">
+      <c r="A19" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>284</v>
+      </c>
+      <c r="E19" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F19" s="3" t="s">
+        <v>285</v>
+      </c>
+      <c r="G19" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="H19" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="I19" s="3" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="20" ht="30" customHeight="1" spans="1:9">
+      <c r="A20" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>286</v>
+      </c>
+      <c r="E20" s="3" t="s">
+        <v>253</v>
+      </c>
+      <c r="F20" s="3" t="s">
+        <v>287</v>
+      </c>
+      <c r="G20" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="H20" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="I20" s="3" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="21" ht="34" spans="1:9">
+      <c r="A21" s="3" t="s">
+        <v>288</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>289</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>290</v>
+      </c>
+      <c r="D21" s="3" t="s">
+        <v>244</v>
+      </c>
+      <c r="E21" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="F21" s="3" t="s">
+        <v>245</v>
+      </c>
+      <c r="G21" s="3" t="s">
+        <v>291</v>
+      </c>
+      <c r="H21" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="I21" s="3" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="22" ht="30" customHeight="1" spans="1:9">
+      <c r="A22" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="D22" s="3" t="s">
+        <v>250</v>
+      </c>
+      <c r="E22" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F22" s="3" t="s">
+        <v>251</v>
+      </c>
+      <c r="G22" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="H22" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="I22" s="3" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="23" ht="30" customHeight="1" spans="1:9">
+      <c r="A23" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="D23" s="3" t="s">
+        <v>252</v>
+      </c>
+      <c r="E23" s="3" t="s">
+        <v>253</v>
+      </c>
+      <c r="F23" s="3" t="s">
+        <v>254</v>
+      </c>
+      <c r="G23" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="H23" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="I23" s="3" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="24" ht="30" customHeight="1" spans="1:9">
+      <c r="A24" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="D24" s="3" t="s">
+        <v>255</v>
+      </c>
+      <c r="E24" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F24" s="3" t="s">
+        <v>256</v>
+      </c>
+      <c r="G24" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="H24" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="I24" s="3" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="25" ht="30" customHeight="1" spans="1:9">
+      <c r="A25" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="D25" s="3" t="s">
+        <v>257</v>
+      </c>
+      <c r="E25" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F25" s="3" t="s">
+        <v>258</v>
+      </c>
+      <c r="G25" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="H25" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="I25" s="3" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="26" ht="30" customHeight="1" spans="1:9">
+      <c r="A26" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="D26" s="3" t="s">
+        <v>259</v>
+      </c>
+      <c r="E26" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F26" s="3" t="s">
+        <v>260</v>
+      </c>
+      <c r="G26" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="H26" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="I26" s="3" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="27" ht="30" customHeight="1" spans="1:9">
+      <c r="A27" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="B27" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="D27" s="3" t="s">
+        <v>261</v>
+      </c>
+      <c r="E27" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F27" s="3" t="s">
+        <v>262</v>
+      </c>
+      <c r="G27" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="H27" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="I27" s="3" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="28" ht="30" customHeight="1" spans="1:9">
+      <c r="A28" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="B28" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="D28" s="3" t="s">
+        <v>263</v>
+      </c>
+      <c r="E28" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="F28" s="3" t="s">
+        <v>264</v>
+      </c>
+      <c r="G28" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="H28" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="I28" s="3" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="29" ht="30" customHeight="1" spans="1:9">
+      <c r="A29" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="B29" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="C29" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="D29" s="3" t="s">
+        <v>265</v>
+      </c>
+      <c r="E29" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F29" s="3" t="s">
+        <v>266</v>
+      </c>
+      <c r="G29" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="H29" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="I29" s="3" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="30" ht="30" customHeight="1" spans="1:9">
+      <c r="A30" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="B30" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="C30" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="D30" s="3" t="s">
+        <v>267</v>
+      </c>
+      <c r="E30" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="F30" s="3" t="s">
+        <v>268</v>
+      </c>
+      <c r="G30" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="H30" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="I30" s="3" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="31" ht="30" customHeight="1" spans="1:9">
+      <c r="A31" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="B31" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="C31" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="D31" s="3" t="s">
+        <v>269</v>
+      </c>
+      <c r="E31" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="F31" s="3" t="s">
+        <v>270</v>
+      </c>
+      <c r="G31" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="H31" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="I31" s="3" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="32" ht="30" customHeight="1" spans="1:9">
+      <c r="A32" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="B32" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="C32" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="D32" s="3" t="s">
+        <v>271</v>
+      </c>
+      <c r="E32" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="F32" s="3" t="s">
+        <v>272</v>
+      </c>
+      <c r="G32" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="H32" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="I32" s="3" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="33" ht="30" customHeight="1" spans="1:9">
+      <c r="A33" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="B33" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="C33" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="D33" s="3" t="s">
+        <v>273</v>
+      </c>
+      <c r="E33" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="F33" s="3" t="s">
+        <v>274</v>
+      </c>
+      <c r="G33" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="H33" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="I33" s="3" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="34" ht="30" customHeight="1" spans="1:9">
+      <c r="A34" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="B34" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="C34" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="D34" s="3" t="s">
+        <v>275</v>
+      </c>
+      <c r="E34" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="F34" s="3" t="s">
+        <v>276</v>
+      </c>
+      <c r="G34" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="H34" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="I34" s="3" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="35" ht="30" customHeight="1" spans="1:9">
+      <c r="A35" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="B35" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="C35" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="D35" s="3" t="s">
+        <v>277</v>
+      </c>
+      <c r="E35" s="3" t="s">
+        <v>278</v>
+      </c>
+      <c r="F35" s="3" t="s">
+        <v>279</v>
+      </c>
+      <c r="G35" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="H35" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="I35" s="3" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="36" ht="30" customHeight="1" spans="1:9">
+      <c r="A36" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="B36" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="C36" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="D36" s="3" t="s">
+        <v>280</v>
+      </c>
+      <c r="E36" s="3" t="s">
+        <v>253</v>
+      </c>
+      <c r="F36" s="3" t="s">
+        <v>281</v>
+      </c>
+      <c r="G36" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="H36" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="I36" s="3" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="37" ht="30" customHeight="1" spans="1:9">
+      <c r="A37" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="B37" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="C37" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="D37" s="3" t="s">
+        <v>282</v>
+      </c>
+      <c r="E37" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F37" s="3" t="s">
+        <v>283</v>
+      </c>
+      <c r="G37" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="H37" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="I37" s="3" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="38" ht="30" customHeight="1" spans="1:9">
+      <c r="A38" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="B38" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="C38" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="D38" s="3" t="s">
+        <v>284</v>
+      </c>
+      <c r="E38" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F38" s="3" t="s">
+        <v>285</v>
+      </c>
+      <c r="G38" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="H38" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="I38" s="3" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="39" ht="30" customHeight="1" spans="1:9">
+      <c r="A39" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="B39" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="C39" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="D39" s="3" t="s">
+        <v>286</v>
+      </c>
+      <c r="E39" s="3" t="s">
+        <v>253</v>
+      </c>
+      <c r="F39" s="3" t="s">
+        <v>287</v>
+      </c>
+      <c r="G39" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="H39" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="I39" s="3" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="40" ht="30" customHeight="1" spans="1:9">
+      <c r="A40" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="B40" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="C40" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="D40" s="3" t="s">
+        <v>293</v>
+      </c>
+      <c r="E40" s="3" t="s">
+        <v>253</v>
+      </c>
+      <c r="F40" s="3" t="s">
+        <v>294</v>
+      </c>
+      <c r="G40" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="H40" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="I40" s="3" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="41" ht="30" customHeight="1" spans="1:9">
+      <c r="A41" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="B41" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="C41" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="D41" s="3" t="s">
+        <v>295</v>
+      </c>
+      <c r="E41" s="3" t="s">
+        <v>253</v>
+      </c>
+      <c r="F41" s="3" t="s">
+        <v>296</v>
+      </c>
+      <c r="G41" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="H41" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="I41" s="3" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="42" ht="30" customHeight="1" spans="1:9">
+      <c r="A42" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="B42" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="C42" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="D42" s="3" t="s">
+        <v>297</v>
+      </c>
+      <c r="E42" s="3" t="s">
+        <v>278</v>
+      </c>
+      <c r="F42" s="3" t="s">
+        <v>298</v>
+      </c>
+      <c r="G42" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="H42" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="I42" s="3" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="43" ht="30" customHeight="1" spans="1:9">
+      <c r="A43" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="B43" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="C43" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="D43" s="3" t="s">
+        <v>299</v>
+      </c>
+      <c r="E43" s="3" t="s">
+        <v>278</v>
+      </c>
+      <c r="F43" s="3" t="s">
+        <v>300</v>
+      </c>
+      <c r="G43" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="H43" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="I43" s="3" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="44" ht="30" customHeight="1" spans="1:9">
+      <c r="A44" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="B44" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="C44" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="D44" s="3" t="s">
+        <v>301</v>
+      </c>
+      <c r="E44" s="3" t="s">
+        <v>278</v>
+      </c>
+      <c r="F44" s="3" t="s">
+        <v>302</v>
+      </c>
+      <c r="G44" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="H44" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="I44" s="3" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="45" ht="30" customHeight="1" spans="1:9">
+      <c r="A45" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="B45" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="C45" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="D45" s="3" t="s">
+        <v>303</v>
+      </c>
+      <c r="E45" s="3" t="s">
+        <v>278</v>
+      </c>
+      <c r="F45" s="3" t="s">
+        <v>304</v>
+      </c>
+      <c r="G45" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="H45" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="I45" s="3" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="46" ht="34" spans="1:9">
+      <c r="A46" s="3" t="s">
+        <v>305</v>
+      </c>
+      <c r="B46" s="3" t="s">
+        <v>306</v>
+      </c>
+      <c r="C46" s="3" t="s">
+        <v>307</v>
+      </c>
+      <c r="D46" s="3" t="s">
+        <v>244</v>
+      </c>
+      <c r="E46" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="F46" s="3" t="s">
+        <v>245</v>
+      </c>
+      <c r="G46" s="3" t="s">
+        <v>308</v>
+      </c>
+      <c r="H46" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="I46" s="3" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="47" ht="30" customHeight="1" spans="1:9">
+      <c r="A47" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="B47" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="C47" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="D47" s="3" t="s">
+        <v>250</v>
+      </c>
+      <c r="E47" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F47" s="3" t="s">
+        <v>251</v>
+      </c>
+      <c r="G47" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="H47" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="I47" s="3" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="48" ht="30" customHeight="1" spans="1:9">
+      <c r="A48" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="B48" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="C48" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="D48" s="3" t="s">
+        <v>252</v>
+      </c>
+      <c r="E48" s="3" t="s">
+        <v>253</v>
+      </c>
+      <c r="F48" s="3" t="s">
+        <v>254</v>
+      </c>
+      <c r="G48" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="H48" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="I48" s="3" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="49" ht="30" customHeight="1" spans="1:9">
+      <c r="A49" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="B49" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="C49" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="D49" s="3" t="s">
+        <v>255</v>
+      </c>
+      <c r="E49" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F49" s="3" t="s">
+        <v>256</v>
+      </c>
+      <c r="G49" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="H49" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="I49" s="3" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="50" ht="30" customHeight="1" spans="1:9">
+      <c r="A50" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="B50" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="C50" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="D50" s="3" t="s">
+        <v>257</v>
+      </c>
+      <c r="E50" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F50" s="3" t="s">
+        <v>258</v>
+      </c>
+      <c r="G50" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="H50" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="I50" s="3" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="51" ht="30" customHeight="1" spans="1:9">
+      <c r="A51" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="B51" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="C51" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="D51" s="3" t="s">
+        <v>259</v>
+      </c>
+      <c r="E51" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F51" s="3" t="s">
+        <v>260</v>
+      </c>
+      <c r="G51" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="H51" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="I51" s="3" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="52" ht="30" customHeight="1" spans="1:9">
+      <c r="A52" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="B52" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="C52" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="D52" s="3" t="s">
+        <v>261</v>
+      </c>
+      <c r="E52" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F52" s="3" t="s">
+        <v>262</v>
+      </c>
+      <c r="G52" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="H52" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="I52" s="3" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="53" ht="30" customHeight="1" spans="1:9">
+      <c r="A53" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="B53" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="C53" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="D53" s="3" t="s">
+        <v>263</v>
+      </c>
+      <c r="E53" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="F53" s="3" t="s">
+        <v>264</v>
+      </c>
+      <c r="G53" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="H53" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="I53" s="3" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="54" ht="30" customHeight="1" spans="1:9">
+      <c r="A54" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="B54" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="C54" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="D54" s="3" t="s">
+        <v>265</v>
+      </c>
+      <c r="E54" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F54" s="3" t="s">
+        <v>266</v>
+      </c>
+      <c r="G54" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="H54" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="I54" s="3" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="55" ht="30" customHeight="1" spans="1:9">
+      <c r="A55" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="B55" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="C55" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="D55" s="3" t="s">
+        <v>267</v>
+      </c>
+      <c r="E55" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="F55" s="3" t="s">
+        <v>268</v>
+      </c>
+      <c r="G55" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="H55" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="I55" s="3" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="56" ht="30" customHeight="1" spans="1:9">
+      <c r="A56" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="B56" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="C56" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="D56" s="3" t="s">
+        <v>269</v>
+      </c>
+      <c r="E56" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="F56" s="3" t="s">
+        <v>270</v>
+      </c>
+      <c r="G56" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="H56" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="I56" s="3" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="57" ht="30" customHeight="1" spans="1:9">
+      <c r="A57" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="B57" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="C57" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="D57" s="3" t="s">
+        <v>271</v>
+      </c>
+      <c r="E57" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="F57" s="3" t="s">
+        <v>272</v>
+      </c>
+      <c r="G57" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="H57" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="I57" s="3" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="58" ht="30" customHeight="1" spans="1:9">
+      <c r="A58" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="B58" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="C58" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="D58" s="3" t="s">
+        <v>273</v>
+      </c>
+      <c r="E58" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="F58" s="3" t="s">
+        <v>274</v>
+      </c>
+      <c r="G58" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="H58" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="I58" s="3" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="59" ht="30" customHeight="1" spans="1:9">
+      <c r="A59" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="B59" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="C59" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="D59" s="3" t="s">
+        <v>275</v>
+      </c>
+      <c r="E59" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="F59" s="3" t="s">
+        <v>276</v>
+      </c>
+      <c r="G59" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="H59" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="I59" s="3" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="60" ht="30" customHeight="1" spans="1:9">
+      <c r="A60" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="B60" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="C60" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="D60" s="3" t="s">
+        <v>277</v>
+      </c>
+      <c r="E60" s="3" t="s">
+        <v>278</v>
+      </c>
+      <c r="F60" s="3" t="s">
+        <v>279</v>
+      </c>
+      <c r="G60" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="H60" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="I60" s="3" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="61" ht="30" customHeight="1" spans="1:9">
+      <c r="A61" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="B61" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="C61" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="D61" s="3" t="s">
+        <v>280</v>
+      </c>
+      <c r="E61" s="3" t="s">
+        <v>253</v>
+      </c>
+      <c r="F61" s="3" t="s">
+        <v>281</v>
+      </c>
+      <c r="G61" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="H61" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="I61" s="3" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="62" ht="30" customHeight="1" spans="1:9">
+      <c r="A62" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="B62" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="C62" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="D62" s="3" t="s">
+        <v>282</v>
+      </c>
+      <c r="E62" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F62" s="3" t="s">
+        <v>283</v>
+      </c>
+      <c r="G62" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="H62" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="I62" s="3" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="63" ht="30" customHeight="1" spans="1:9">
+      <c r="A63" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="B63" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="C63" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="D63" s="3" t="s">
+        <v>284</v>
+      </c>
+      <c r="E63" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F63" s="3" t="s">
+        <v>285</v>
+      </c>
+      <c r="G63" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="H63" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="I63" s="3" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="64" ht="30" customHeight="1" spans="1:9">
+      <c r="A64" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="B64" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="C64" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="D64" s="3" t="s">
+        <v>286</v>
+      </c>
+      <c r="E64" s="3" t="s">
+        <v>253</v>
+      </c>
+      <c r="F64" s="3" t="s">
+        <v>287</v>
+      </c>
+      <c r="G64" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="H64" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="I64" s="3" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="65" ht="30" customHeight="1" spans="1:9">
+      <c r="A65" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="B65" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="C65" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="D65" s="3" t="s">
+        <v>310</v>
+      </c>
+      <c r="E65" s="3" t="s">
+        <v>253</v>
+      </c>
+      <c r="F65" s="3" t="s">
+        <v>311</v>
+      </c>
+      <c r="G65" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="H65" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="I65" s="3" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="66" ht="30" customHeight="1" spans="1:9">
+      <c r="A66" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="B66" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="C66" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="D66" s="3" t="s">
+        <v>312</v>
+      </c>
+      <c r="E66" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="F66" s="3" t="s">
+        <v>313</v>
+      </c>
+      <c r="G66" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="H66" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="I66" s="3" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="67" ht="30" customHeight="1" spans="1:9">
+      <c r="A67" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="B67" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="C67" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="D67" s="3" t="s">
+        <v>314</v>
+      </c>
+      <c r="E67" s="3" t="s">
+        <v>315</v>
+      </c>
+      <c r="F67" s="3" t="s">
+        <v>316</v>
+      </c>
+      <c r="G67" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="H67" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="I67" s="3" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="68" ht="30" customHeight="1" spans="1:9">
+      <c r="A68" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="B68" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="C68" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="D68" s="3" t="s">
+        <v>317</v>
+      </c>
+      <c r="E68" s="3" t="s">
+        <v>278</v>
+      </c>
+      <c r="F68" s="3" t="s">
+        <v>318</v>
+      </c>
+      <c r="G68" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="H68" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="I68" s="3" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="69" ht="30" customHeight="1" spans="1:9">
+      <c r="A69" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="B69" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="C69" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="D69" s="3" t="s">
+        <v>293</v>
+      </c>
+      <c r="E69" s="3" t="s">
+        <v>253</v>
+      </c>
+      <c r="F69" s="3" t="s">
+        <v>319</v>
+      </c>
+      <c r="G69" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="H69" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="I69" s="3" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="70" ht="30" customHeight="1" spans="1:9">
+      <c r="A70" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="B70" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="C70" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="D70" s="3" t="s">
+        <v>295</v>
+      </c>
+      <c r="E70" s="3" t="s">
+        <v>253</v>
+      </c>
+      <c r="F70" s="3" t="s">
+        <v>320</v>
+      </c>
+      <c r="G70" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="H70" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="I70" s="3" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="71" ht="30" customHeight="1" spans="1:9">
+      <c r="A71" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="B71" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="C71" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="D71" s="3" t="s">
+        <v>297</v>
+      </c>
+      <c r="E71" s="3" t="s">
+        <v>278</v>
+      </c>
+      <c r="F71" s="3" t="s">
+        <v>321</v>
+      </c>
+      <c r="G71" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="H71" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="I71" s="3" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="72" ht="30" customHeight="1" spans="1:9">
+      <c r="A72" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="B72" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="C72" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="D72" s="3" t="s">
+        <v>299</v>
+      </c>
+      <c r="E72" s="3" t="s">
+        <v>278</v>
+      </c>
+      <c r="F72" s="3" t="s">
+        <v>322</v>
+      </c>
+      <c r="G72" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="H72" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="I72" s="3" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="73" ht="30" customHeight="1" spans="1:9">
+      <c r="A73" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="B73" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="C73" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="D73" s="3" t="s">
+        <v>301</v>
+      </c>
+      <c r="E73" s="3" t="s">
+        <v>278</v>
+      </c>
+      <c r="F73" s="3" t="s">
+        <v>323</v>
+      </c>
+      <c r="G73" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="H73" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="I73" s="3" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="74" ht="30" customHeight="1" spans="1:9">
+      <c r="A74" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="B74" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="C74" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="D74" s="3" t="s">
+        <v>303</v>
+      </c>
+      <c r="E74" s="3" t="s">
+        <v>278</v>
+      </c>
+      <c r="F74" s="3" t="s">
+        <v>324</v>
+      </c>
+      <c r="G74" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="H74" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="I74" s="3" t="s">
+        <v>249</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:I74" etc:filterBottomFollowUsedRange="0">
+    <extLst/>
+  </autoFilter>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
 </file>
</xml_diff>